<commit_message>
Added Novelty no reset with landmarks tiebreaker
</commit_message>
<xml_diff>
--- a/Tests/Evaluation/Experiment/Strategy List.xlsx
+++ b/Tests/Evaluation/Experiment/Strategy List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Cael\Documents\University files\4th Year\Dissertation\4th-Year-Dissertation\Tests\Evaluation\Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5E647D0-9620-4E56-AC6A-E785C9274054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADBA059-101B-4BA1-9B14-A86F8E1F5CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36C2E955-2634-424C-8826-53A49E0BD8E3}"/>
   </bookViews>
@@ -601,7 +601,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="2" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Landmarks with Tree Distance tiebreaker
</commit_message>
<xml_diff>
--- a/Tests/Evaluation/Experiment/Strategy List.xlsx
+++ b/Tests/Evaluation/Experiment/Strategy List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Cael\Documents\University files\4th Year\Dissertation\4th-Year-Dissertation\Tests\Evaluation\Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADBA059-101B-4BA1-9B14-A86F8E1F5CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD614D7E-5535-4629-9D9E-6F0B5614FEE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36C2E955-2634-424C-8826-53A49E0BD8E3}"/>
   </bookViews>
@@ -535,7 +535,7 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -549,7 +549,7 @@
       <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Landmarks Newest First
</commit_message>
<xml_diff>
--- a/Tests/Evaluation/Experiment/Strategy List.xlsx
+++ b/Tests/Evaluation/Experiment/Strategy List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Cael\Documents\University files\4th Year\Dissertation\4th-Year-Dissertation\Tests\Evaluation\Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD614D7E-5535-4629-9D9E-6F0B5614FEE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9EBC6B1-E59A-48A8-99B1-FE8388112E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36C2E955-2634-424C-8826-53A49E0BD8E3}"/>
   </bookViews>
@@ -563,7 +563,7 @@
       <c r="D4" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Hamming Distance with Tree Distance tiebreaker
</commit_message>
<xml_diff>
--- a/Tests/Evaluation/Experiment/Strategy List.xlsx
+++ b/Tests/Evaluation/Experiment/Strategy List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Cael\Documents\University files\4th Year\Dissertation\4th-Year-Dissertation\Tests\Evaluation\Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9EBC6B1-E59A-48A8-99B1-FE8388112E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5478B33-EF53-4FE3-8ECE-2E0B2BECA453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36C2E955-2634-424C-8826-53A49E0BD8E3}"/>
   </bookViews>
@@ -554,7 +554,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C4" t="s">

</xml_diff>

<commit_message>
Added Tree Distance with Landmarks tiebreaker
</commit_message>
<xml_diff>
--- a/Tests/Evaluation/Experiment/Strategy List.xlsx
+++ b/Tests/Evaluation/Experiment/Strategy List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Cael\Documents\University files\4th Year\Dissertation\4th-Year-Dissertation\Tests\Evaluation\Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5478B33-EF53-4FE3-8ECE-2E0B2BECA453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6849F767-4AC6-4C93-A88B-5BC92AC5004A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36C2E955-2634-424C-8826-53A49E0BD8E3}"/>
   </bookViews>
@@ -568,7 +568,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D5" t="s">

</xml_diff>

<commit_message>
Added Hamming Distance with Landmarks tiebreaker
</commit_message>
<xml_diff>
--- a/Tests/Evaluation/Experiment/Strategy List.xlsx
+++ b/Tests/Evaluation/Experiment/Strategy List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Cael\Documents\University files\4th Year\Dissertation\4th-Year-Dissertation\Tests\Evaluation\Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6849F767-4AC6-4C93-A88B-5BC92AC5004A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B6F9DA9-5938-4DEA-A52F-420B53CBE497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36C2E955-2634-424C-8826-53A49E0BD8E3}"/>
   </bookViews>
@@ -540,7 +540,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C3" t="s">

</xml_diff>

<commit_message>
Added novelty for methods and tasks
</commit_message>
<xml_diff>
--- a/Tests/Evaluation/Experiment/Strategy List.xlsx
+++ b/Tests/Evaluation/Experiment/Strategy List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Cael\Documents\University files\4th Year\Dissertation\4th-Year-Dissertation\Tests\Evaluation\Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B6F9DA9-5938-4DEA-A52F-420B53CBE497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF425064-85EB-411C-A228-80BD8C527E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36C2E955-2634-424C-8826-53A49E0BD8E3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>Hamming Distance Seen States</t>
   </si>
@@ -125,10 +125,19 @@
     <t>Novelty - Methods - Reset</t>
   </si>
   <si>
-    <t>Novelty Level 1 - With Methods &amp; Tasks - Reset</t>
-  </si>
-  <si>
     <t>Landmarks newest First</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novelty Level 1 - With Methods &amp; Tasks </t>
+  </si>
+  <si>
+    <t>Novelty Level 1 - With Methods &amp; Tasks - oldest First</t>
+  </si>
+  <si>
+    <t>Novelty Level 1 - With Methods - No Reset - oldest first</t>
+  </si>
+  <si>
+    <t>Novelty Level 1 - With Methods - Reset - oldest first</t>
   </si>
 </sst>
 </file>
@@ -564,7 +573,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -621,21 +630,33 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D15" s="1" t="s">
-        <v>29</v>
+      <c r="D15" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D16" s="1"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Removed Novelty methods with no reset. Added novelty methods oldest first
</commit_message>
<xml_diff>
--- a/Tests/Evaluation/Experiment/Strategy List.xlsx
+++ b/Tests/Evaluation/Experiment/Strategy List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Cael\Documents\University files\4th Year\Dissertation\4th-Year-Dissertation\Tests\Evaluation\Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF425064-85EB-411C-A228-80BD8C527E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B0A193-D67C-448B-A537-328F74BE67C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36C2E955-2634-424C-8826-53A49E0BD8E3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Hamming Distance Seen States</t>
   </si>
@@ -101,9 +101,6 @@
     <t>Landmarks with Tree Distance Tie Breaker</t>
   </si>
   <si>
-    <t xml:space="preserve">Novelty Level 1 - With Methods - No Reset </t>
-  </si>
-  <si>
     <t>Novelty Level 1 - Reset - Landmarks Tie Breaker</t>
   </si>
   <si>
@@ -132,9 +129,6 @@
   </si>
   <si>
     <t>Novelty Level 1 - With Methods &amp; Tasks - oldest First</t>
-  </si>
-  <si>
-    <t>Novelty Level 1 - With Methods - No Reset - oldest first</t>
   </si>
   <si>
     <t>Novelty Level 1 - With Methods - Reset - oldest first</t>
@@ -186,9 +180,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -530,7 +523,7 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
@@ -544,12 +537,12 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C3" t="s">
@@ -558,12 +551,12 @@
       <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C4" t="s">
@@ -572,16 +565,16 @@
       <c r="D4" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>29</v>
+      <c r="E4" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -595,42 +588,42 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D14" s="2" t="s">
-        <v>25</v>
+      <c r="D14" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="1" t="s">
         <v>30</v>
       </c>
     </row>
@@ -639,29 +632,19 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D17" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Modified novelty state calculation
</commit_message>
<xml_diff>
--- a/Tests/Evaluation/Experiment/Strategy List.xlsx
+++ b/Tests/Evaluation/Experiment/Strategy List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Cael\Documents\University files\4th Year\Dissertation\4th-Year-Dissertation\Tests\Evaluation\Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B0A193-D67C-448B-A537-328F74BE67C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39074A04-AB7B-48CB-8D90-856064D8EADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36C2E955-2634-424C-8826-53A49E0BD8E3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Hamming Distance Seen States</t>
   </si>
@@ -132,6 +132,9 @@
   </si>
   <si>
     <t>Novelty Level 1 - With Methods - Reset - oldest first</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -500,7 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A62831C5-BE86-482F-892C-884E40B5F8BA}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
@@ -632,19 +635,24 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>32</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Failed strategies ready for rerun
</commit_message>
<xml_diff>
--- a/Tests/Evaluation/Experiment/Strategy List.xlsx
+++ b/Tests/Evaluation/Experiment/Strategy List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Cael\Documents\University files\4th Year\Dissertation\4th-Year-Dissertation\Tests\Evaluation\Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63BE4192-DB0B-4ADF-8962-1DA6472FCA22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268DADFE-D18F-4153-9BDF-83B7FC987583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36C2E955-2634-424C-8826-53A49E0BD8E3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="31">
   <si>
     <t>Hamming Distance Seen States</t>
   </si>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>WAITING</t>
   </si>
   <si>
     <t>RUNNING</t>
@@ -138,7 +135,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -148,13 +145,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -187,11 +177,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -524,8 +513,8 @@
       <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>31</v>
+      <c r="C1" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -535,8 +524,8 @@
       <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>31</v>
+      <c r="C2" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -546,8 +535,8 @@
       <c r="B3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>31</v>
+      <c r="C3" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="G3" s="1"/>
     </row>
@@ -558,8 +547,8 @@
       <c r="B4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>31</v>
+      <c r="C4" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -569,8 +558,8 @@
       <c r="B5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>31</v>
+      <c r="C5" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -580,8 +569,8 @@
       <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>31</v>
+      <c r="C6" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -591,8 +580,8 @@
       <c r="B7" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>31</v>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -602,8 +591,8 @@
       <c r="B8" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>31</v>
+      <c r="C8" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -613,8 +602,8 @@
       <c r="B9" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>31</v>
+      <c r="C9" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -624,8 +613,8 @@
       <c r="B10" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>31</v>
+      <c r="C10" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -635,8 +624,8 @@
       <c r="B11" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>31</v>
+      <c r="C11" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -646,8 +635,8 @@
       <c r="B12" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>31</v>
+      <c r="C12" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -657,8 +646,8 @@
       <c r="B13" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>31</v>
+      <c r="C13" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -679,8 +668,8 @@
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>31</v>
+      <c r="C15" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -690,8 +679,8 @@
       <c r="B16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>31</v>
+      <c r="C16" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -701,8 +690,8 @@
       <c r="B17" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>31</v>
+      <c r="C17" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -712,8 +701,8 @@
       <c r="B18" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>31</v>
+      <c r="C18" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -723,8 +712,8 @@
       <c r="B19" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>31</v>
+      <c r="C19" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -792,8 +781,8 @@
       <c r="B25" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>31</v>
+      <c r="C25" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -825,8 +814,8 @@
       <c r="B28" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>31</v>
+      <c r="C28" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -836,8 +825,8 @@
       <c r="B29" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>31</v>
+      <c r="C29" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>